<commit_message>
Criação do arquivo para testar erros.
</commit_message>
<xml_diff>
--- a/meus_testes/test/lista_test.xlsx
+++ b/meus_testes/test/lista_test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20343"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENAI\Desktop\teste_sf\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENAI\Desktop\teste_sf\meus_testes\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9712D910-D2A3-4D76-BEA7-384F0CD462B9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D00243C5-2755-4B7C-A3CA-3559DA48A9F1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="88">
   <si>
     <t>HAPPY_PATH</t>
   </si>
@@ -279,10 +279,13 @@
     <t>Testando uma lista com string e número.</t>
   </si>
   <si>
-    <t>[8, "note", 5]</t>
-  </si>
-  <si>
     <t>Testando um número sem uma lista.</t>
+  </si>
+  <si>
+    <t>[8, "nove", 5]</t>
+  </si>
+  <si>
+    <t>TypeError("A lista de notas não pode estar vazia")</t>
   </si>
 </sst>
 </file>
@@ -1774,7 +1777,7 @@
         <v>83</v>
       </c>
       <c r="E16" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1822,7 +1825,7 @@
         <v>84</v>
       </c>
       <c r="D19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E19" t="s">
         <v>75</v>
@@ -1836,7 +1839,7 @@
         <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D20">
         <v>8</v>

</xml_diff>